<commit_message>
feat: enrich medication references in pseudonym snapshots refs #1264
</commit_message>
<xml_diff>
--- a/R-cds2db/cds2db/inst/extdata/Table_Description_Definition.xlsx
+++ b/R-cds2db/cds2db/inst/extdata/Table_Description_Definition.xlsx
@@ -3463,7 +3463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" style="12" min="1" max="1"/>
@@ -3638,6 +3638,168 @@
         </is>
       </c>
       <c r="E10" s="19" t="inlineStr">
+        <is>
+          <t>keep</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="19" t="inlineStr">
+        <is>
+          <t>medicationrequest</t>
+        </is>
+      </c>
+      <c r="B11" s="19" t="inlineStr">
+        <is>
+          <t>medreq_medication_system</t>
+        </is>
+      </c>
+      <c r="C11" s="19" t="inlineStr">
+        <is>
+          <t>Codesystem der referenzierten Medication</t>
+        </is>
+      </c>
+      <c r="D11" s="19" t="inlineStr">
+        <is>
+          <t>varchar</t>
+        </is>
+      </c>
+      <c r="E11" s="19" t="inlineStr">
+        <is>
+          <t>keep</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="19" t="inlineStr">
+        <is>
+          <t>medicationrequest</t>
+        </is>
+      </c>
+      <c r="B12" s="19" t="inlineStr">
+        <is>
+          <t>medreq_medication_code</t>
+        </is>
+      </c>
+      <c r="C12" s="19" t="inlineStr">
+        <is>
+          <t>Code der referenzierten Medication</t>
+        </is>
+      </c>
+      <c r="D12" s="19" t="inlineStr">
+        <is>
+          <t>varchar</t>
+        </is>
+      </c>
+      <c r="E12" s="19" t="inlineStr">
+        <is>
+          <t>keep</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="19" t="inlineStr">
+        <is>
+          <t>medicationadministration</t>
+        </is>
+      </c>
+      <c r="B13" s="19" t="inlineStr">
+        <is>
+          <t>medadm_medication_system</t>
+        </is>
+      </c>
+      <c r="C13" s="19" t="inlineStr">
+        <is>
+          <t>Codesystem der referenzierten Medication</t>
+        </is>
+      </c>
+      <c r="D13" s="19" t="inlineStr">
+        <is>
+          <t>varchar</t>
+        </is>
+      </c>
+      <c r="E13" s="19" t="inlineStr">
+        <is>
+          <t>keep</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="19" t="inlineStr">
+        <is>
+          <t>medicationadministration</t>
+        </is>
+      </c>
+      <c r="B14" s="19" t="inlineStr">
+        <is>
+          <t>medadm_medication_code</t>
+        </is>
+      </c>
+      <c r="C14" s="19" t="inlineStr">
+        <is>
+          <t>Code der referenzierten Medication</t>
+        </is>
+      </c>
+      <c r="D14" s="19" t="inlineStr">
+        <is>
+          <t>varchar</t>
+        </is>
+      </c>
+      <c r="E14" s="19" t="inlineStr">
+        <is>
+          <t>keep</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="19" t="inlineStr">
+        <is>
+          <t>medicationstatement</t>
+        </is>
+      </c>
+      <c r="B15" s="19" t="inlineStr">
+        <is>
+          <t>medstat_medication_system</t>
+        </is>
+      </c>
+      <c r="C15" s="19" t="inlineStr">
+        <is>
+          <t>Codesystem der referenzierten Medication</t>
+        </is>
+      </c>
+      <c r="D15" s="19" t="inlineStr">
+        <is>
+          <t>varchar</t>
+        </is>
+      </c>
+      <c r="E15" s="19" t="inlineStr">
+        <is>
+          <t>keep</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="19" t="inlineStr">
+        <is>
+          <t>medicationstatement</t>
+        </is>
+      </c>
+      <c r="B16" s="19" t="inlineStr">
+        <is>
+          <t>medstat_medication_code</t>
+        </is>
+      </c>
+      <c r="C16" s="19" t="inlineStr">
+        <is>
+          <t>Code der referenzierten Medication</t>
+        </is>
+      </c>
+      <c r="D16" s="19" t="inlineStr">
+        <is>
+          <t>varchar</t>
+        </is>
+      </c>
+      <c r="E16" s="19" t="inlineStr">
         <is>
           <t>keep</t>
         </is>

</xml_diff>

<commit_message>
revert: remove observation LOINC enrichment refs #1264
</commit_message>
<xml_diff>
--- a/R-cds2db/cds2db/inst/extdata/Table_Description_Definition.xlsx
+++ b/R-cds2db/cds2db/inst/extdata/Table_Description_Definition.xlsx
@@ -3463,7 +3463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" style="12" min="1" max="1"/>
@@ -3565,22 +3565,22 @@
     <row r="8" s="12">
       <c r="A8" s="19" t="inlineStr">
         <is>
-          <t>observation</t>
+          <t>medicationrequest</t>
         </is>
       </c>
       <c r="B8" s="19" t="inlineStr">
         <is>
-          <t>value_in_reference_unit</t>
+          <t>medreq_medication_system</t>
         </is>
       </c>
       <c r="C8" s="19" t="inlineStr">
         <is>
-          <t>Wert in Referenzeinheit</t>
+          <t>Codesystem der referenzierten Medication</t>
         </is>
       </c>
       <c r="D8" s="19" t="inlineStr">
         <is>
-          <t>double precision</t>
+          <t>varchar</t>
         </is>
       </c>
       <c r="E8" s="19" t="inlineStr">
@@ -3592,17 +3592,17 @@
     <row r="9">
       <c r="A9" s="19" t="inlineStr">
         <is>
-          <t>observation</t>
+          <t>medicationrequest</t>
         </is>
       </c>
       <c r="B9" s="19" t="inlineStr">
         <is>
-          <t>reference_unit</t>
+          <t>medreq_medication_code</t>
         </is>
       </c>
       <c r="C9" s="19" t="inlineStr">
         <is>
-          <t>Referenzeinheit</t>
+          <t>Code der referenzierten Medication</t>
         </is>
       </c>
       <c r="D9" s="19" t="inlineStr">
@@ -3619,17 +3619,17 @@
     <row r="10">
       <c r="A10" s="19" t="inlineStr">
         <is>
-          <t>observation</t>
+          <t>medicationadministration</t>
         </is>
       </c>
       <c r="B10" s="19" t="inlineStr">
         <is>
-          <t>primary_loinc_code</t>
+          <t>medadm_medication_system</t>
         </is>
       </c>
       <c r="C10" s="19" t="inlineStr">
         <is>
-          <t>Primary LOINC Code</t>
+          <t>Codesystem der referenzierten Medication</t>
         </is>
       </c>
       <c r="D10" s="19" t="inlineStr">
@@ -3646,17 +3646,17 @@
     <row r="11">
       <c r="A11" s="19" t="inlineStr">
         <is>
-          <t>medicationrequest</t>
+          <t>medicationadministration</t>
         </is>
       </c>
       <c r="B11" s="19" t="inlineStr">
         <is>
-          <t>medreq_medication_system</t>
+          <t>medadm_medication_code</t>
         </is>
       </c>
       <c r="C11" s="19" t="inlineStr">
         <is>
-          <t>Codesystem der referenzierten Medication</t>
+          <t>Code der referenzierten Medication</t>
         </is>
       </c>
       <c r="D11" s="19" t="inlineStr">
@@ -3673,17 +3673,17 @@
     <row r="12">
       <c r="A12" s="19" t="inlineStr">
         <is>
-          <t>medicationrequest</t>
+          <t>medicationstatement</t>
         </is>
       </c>
       <c r="B12" s="19" t="inlineStr">
         <is>
-          <t>medreq_medication_code</t>
+          <t>medstat_medication_system</t>
         </is>
       </c>
       <c r="C12" s="19" t="inlineStr">
         <is>
-          <t>Code der referenzierten Medication</t>
+          <t>Codesystem der referenzierten Medication</t>
         </is>
       </c>
       <c r="D12" s="19" t="inlineStr">
@@ -3700,17 +3700,17 @@
     <row r="13">
       <c r="A13" s="19" t="inlineStr">
         <is>
-          <t>medicationadministration</t>
+          <t>medicationstatement</t>
         </is>
       </c>
       <c r="B13" s="19" t="inlineStr">
         <is>
-          <t>medadm_medication_system</t>
+          <t>medstat_medication_code</t>
         </is>
       </c>
       <c r="C13" s="19" t="inlineStr">
         <is>
-          <t>Codesystem der referenzierten Medication</t>
+          <t>Code der referenzierten Medication</t>
         </is>
       </c>
       <c r="D13" s="19" t="inlineStr">
@@ -3719,87 +3719,6 @@
         </is>
       </c>
       <c r="E13" s="19" t="inlineStr">
-        <is>
-          <t>keep</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="19" t="inlineStr">
-        <is>
-          <t>medicationadministration</t>
-        </is>
-      </c>
-      <c r="B14" s="19" t="inlineStr">
-        <is>
-          <t>medadm_medication_code</t>
-        </is>
-      </c>
-      <c r="C14" s="19" t="inlineStr">
-        <is>
-          <t>Code der referenzierten Medication</t>
-        </is>
-      </c>
-      <c r="D14" s="19" t="inlineStr">
-        <is>
-          <t>varchar</t>
-        </is>
-      </c>
-      <c r="E14" s="19" t="inlineStr">
-        <is>
-          <t>keep</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="19" t="inlineStr">
-        <is>
-          <t>medicationstatement</t>
-        </is>
-      </c>
-      <c r="B15" s="19" t="inlineStr">
-        <is>
-          <t>medstat_medication_system</t>
-        </is>
-      </c>
-      <c r="C15" s="19" t="inlineStr">
-        <is>
-          <t>Codesystem der referenzierten Medication</t>
-        </is>
-      </c>
-      <c r="D15" s="19" t="inlineStr">
-        <is>
-          <t>varchar</t>
-        </is>
-      </c>
-      <c r="E15" s="19" t="inlineStr">
-        <is>
-          <t>keep</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="19" t="inlineStr">
-        <is>
-          <t>medicationstatement</t>
-        </is>
-      </c>
-      <c r="B16" s="19" t="inlineStr">
-        <is>
-          <t>medstat_medication_code</t>
-        </is>
-      </c>
-      <c r="C16" s="19" t="inlineStr">
-        <is>
-          <t>Code der referenzierten Medication</t>
-        </is>
-      </c>
-      <c r="D16" s="19" t="inlineStr">
-        <is>
-          <t>varchar</t>
-        </is>
-      </c>
-      <c r="E16" s="19" t="inlineStr">
         <is>
           <t>keep</t>
         </is>

</xml_diff>

<commit_message>
feat: enrich and deduplicate snapshots refs #1264
</commit_message>
<xml_diff>
--- a/R-cds2db/cds2db/inst/extdata/Table_Description_Definition.xlsx
+++ b/R-cds2db/cds2db/inst/extdata/Table_Description_Definition.xlsx
@@ -3463,7 +3463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" style="12" min="1" max="1"/>
@@ -3719,6 +3719,60 @@
         </is>
       </c>
       <c r="E13" s="19" t="inlineStr">
+        <is>
+          <t>keep</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="19" t="inlineStr">
+        <is>
+          <t>fall</t>
+        </is>
+      </c>
+      <c r="B14" s="19" t="inlineStr">
+        <is>
+          <t>fall_age_at_admission</t>
+        </is>
+      </c>
+      <c r="C14" s="19" t="inlineStr">
+        <is>
+          <t>Alter bei Aufnahme des Falls in abgeschlossenen Jahren</t>
+        </is>
+      </c>
+      <c r="D14" s="19" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="E14" s="19" t="inlineStr">
+        <is>
+          <t>keep</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="19" t="inlineStr">
+        <is>
+          <t>encounter</t>
+        </is>
+      </c>
+      <c r="B15" s="19" t="inlineStr">
+        <is>
+          <t>enc_age_at_admission</t>
+        </is>
+      </c>
+      <c r="C15" s="19" t="inlineStr">
+        <is>
+          <t>Alter bei Beginn des Encounters in abgeschlossenen Jahren</t>
+        </is>
+      </c>
+      <c r="D15" s="19" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="E15" s="19" t="inlineStr">
         <is>
           <t>keep</t>
         </is>

</xml_diff>

<commit_message>
feat: enrich observations with LOINC reference values refs #1264
</commit_message>
<xml_diff>
--- a/R-cds2db/cds2db/inst/extdata/Table_Description_Definition.xlsx
+++ b/R-cds2db/cds2db/inst/extdata/Table_Description_Definition.xlsx
@@ -3463,7 +3463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" style="12" min="1" max="1"/>
@@ -3773,6 +3773,87 @@
         </is>
       </c>
       <c r="E15" s="19" t="inlineStr">
+        <is>
+          <t>keep</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="19" t="inlineStr">
+        <is>
+          <t>observation</t>
+        </is>
+      </c>
+      <c r="B16" s="19" t="inlineStr">
+        <is>
+          <t>value_in_reference_unit</t>
+        </is>
+      </c>
+      <c r="C16" s="19" t="inlineStr">
+        <is>
+          <t>Observation-Wert in der Referenzeinheit aus der LOINC-Mapping-Tabelle</t>
+        </is>
+      </c>
+      <c r="D16" s="19" t="inlineStr">
+        <is>
+          <t>double</t>
+        </is>
+      </c>
+      <c r="E16" s="19" t="inlineStr">
+        <is>
+          <t>keep</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="19" t="inlineStr">
+        <is>
+          <t>observation</t>
+        </is>
+      </c>
+      <c r="B17" s="19" t="inlineStr">
+        <is>
+          <t>reference_unit</t>
+        </is>
+      </c>
+      <c r="C17" s="19" t="inlineStr">
+        <is>
+          <t>Referenzeinheit aus der LOINC-Mapping-Tabelle</t>
+        </is>
+      </c>
+      <c r="D17" s="19" t="inlineStr">
+        <is>
+          <t>varchar</t>
+        </is>
+      </c>
+      <c r="E17" s="19" t="inlineStr">
+        <is>
+          <t>keep</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="19" t="inlineStr">
+        <is>
+          <t>observation</t>
+        </is>
+      </c>
+      <c r="B18" s="19" t="inlineStr">
+        <is>
+          <t>primary_loinc_code</t>
+        </is>
+      </c>
+      <c r="C18" s="19" t="inlineStr">
+        <is>
+          <t>Primärer LOINC aus der LOINC-Mapping-Tabelle</t>
+        </is>
+      </c>
+      <c r="D18" s="19" t="inlineStr">
+        <is>
+          <t>varchar</t>
+        </is>
+      </c>
+      <c r="E18" s="19" t="inlineStr">
         <is>
           <t>keep</t>
         </is>

</xml_diff>